<commit_message>
Readdress email to Josef Srejber; add MW reference CZ26011282
Email is internal to the Maurice Ward rail agent, not direct to Sonavox, so
it asks him to obtain the answers from Sonavox/the shipper.

Summary now records reference CZ26011282, free-circulation procedure,
A1 Ostrava clearance office and week-34 arrival.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThmrE3pZ6fcsX17xx42UdU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonavox_Technology_CZ_TECGO26080029.xlsx
+++ b/output/HS_Code_Summary_Sonavox_Technology_CZ_TECGO26080029.xlsx
@@ -26,9 +26,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="200">
   <si>
     <t xml:space="preserve">HS CODE SUMMARY – Sonavox Technology CZ s.r.o.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference MW:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CZ26011282 (Josef Šrejber – RAIL) | celní režim: volný oběh | celnice: A1 Ostrava | příjezd cca 34. týden</t>
   </si>
   <si>
     <t xml:space="preserve">Odesílatelé / Senders:</t>
@@ -1213,7 +1219,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1315,10 +1321,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1331,581 +1337,573 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="6" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="B18" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="H18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="I18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="L17" s="6" t="s">
+      <c r="J18" s="6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="K18" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="L18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="8" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="B19" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="9" t="n">
-        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A18,'Line items'!$F$2:$F$25,$C18)</f>
-        <v>65000</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A18,'Line items'!$F$2:$F$25,$C18)</f>
-        <v>86.5</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A18,'Line items'!$F$2:$F$25,$C18)</f>
-        <v>216.33</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A18,'Line items'!$F$2:$F$25,$C18)</f>
-        <v>9841</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J18" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L18" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A19,'Line items'!$F$2:$F$25,$C19)</f>
-        <v>778000</v>
+        <v>65000</v>
       </c>
       <c r="F19" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A19,'Line items'!$F$2:$F$25,$C19)</f>
-        <v>8806.4</v>
+        <v>86.5</v>
       </c>
       <c r="G19" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A19,'Line items'!$F$2:$F$25,$C19)</f>
-        <v>8990.91</v>
+        <v>216.33</v>
       </c>
       <c r="H19" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A19,'Line items'!$F$2:$F$25,$C19)</f>
-        <v>32182.14</v>
+        <v>9841</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L19" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>49</v>
       </c>
       <c r="E20" s="9" t="n">
         <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A20,'Line items'!$F$2:$F$25,$C20)</f>
-        <v>9960</v>
+        <v>778000</v>
       </c>
       <c r="F20" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A20,'Line items'!$F$2:$F$25,$C20)</f>
-        <v>103.09</v>
+        <v>8806.4</v>
       </c>
       <c r="G20" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A20,'Line items'!$F$2:$F$25,$C20)</f>
-        <v>128</v>
+        <v>8990.91</v>
       </c>
       <c r="H20" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A20,'Line items'!$F$2:$F$25,$C20)</f>
-        <v>1378.1</v>
+        <v>32182.14</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>52</v>
       </c>
       <c r="E21" s="9" t="n">
         <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A21,'Line items'!$F$2:$F$25,$C21)</f>
-        <v>210000</v>
+        <v>9960</v>
       </c>
       <c r="F21" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A21,'Line items'!$F$2:$F$25,$C21)</f>
-        <v>30.24</v>
+        <v>103.09</v>
       </c>
       <c r="G21" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A21,'Line items'!$F$2:$F$25,$C21)</f>
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="H21" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A21,'Line items'!$F$2:$F$25,$C21)</f>
-        <v>8820</v>
+        <v>1378.1</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L21" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="12" t="s">
+      <c r="D22" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="13" t="n">
+      <c r="E22" s="9" t="n">
         <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
         <v>210000</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="F22" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
+        <v>30.24</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
+        <v>40</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
+        <v>8820</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
+        <v>210000</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
         <v>312.3</v>
       </c>
-      <c r="G22" s="14" t="n">
-        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
+      <c r="G23" s="14" t="n">
+        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
         <v>325.5</v>
       </c>
-      <c r="H22" s="14" t="n">
-        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A22,'Line items'!$F$2:$F$25,$C22)</f>
+      <c r="H23" s="14" t="n">
+        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
         <v>13140</v>
       </c>
-      <c r="I22" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="K22" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="L22" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="8" t="s">
+      <c r="I23" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J23" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="K23" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="L23" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E23" s="9" t="n">
-        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A24,'Line items'!$F$2:$F$25,$C24)</f>
         <v>51200</v>
       </c>
-      <c r="F23" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
+      <c r="F24" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A24,'Line items'!$F$2:$F$25,$C24)</f>
         <v>235.52</v>
       </c>
-      <c r="G23" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
+      <c r="G24" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A24,'Line items'!$F$2:$F$25,$C24)</f>
         <v>250</v>
       </c>
-      <c r="H23" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A23,'Line items'!$F$2:$F$25,$C23)</f>
+      <c r="H24" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A24,'Line items'!$F$2:$F$25,$C24)</f>
         <v>8120.32</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L23" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="E24" s="18" t="n">
-        <f aca="false">SUM(E18:E23)</f>
+      <c r="I24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <f aca="false">SUM(E19:E24)</f>
         <v>1324160</v>
       </c>
-      <c r="F24" s="19" t="n">
-        <f aca="false">SUM(F18:F23)</f>
+      <c r="F25" s="19" t="n">
+        <f aca="false">SUM(F19:F24)</f>
         <v>9574.05</v>
       </c>
-      <c r="G24" s="19" t="n">
-        <f aca="false">SUM(G18:G23)</f>
+      <c r="G25" s="19" t="n">
+        <f aca="false">SUM(G19:G24)</f>
         <v>9950.74</v>
       </c>
-      <c r="H24" s="19" t="n">
-        <f aca="false">SUM(H18:H23)</f>
+      <c r="H25" s="19" t="n">
+        <f aca="false">SUM(H19:H24)</f>
         <v>73481.56</v>
       </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A25,'Line items'!$F$2:$F$25,$C25)</f>
-        <v>19152</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A25,'Line items'!$F$2:$F$25,$C25)</f>
-        <v>11299.68</v>
-      </c>
-      <c r="G25" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A25,'Line items'!$F$2:$F$25,$C25)</f>
-        <v>11688.8</v>
-      </c>
-      <c r="H25" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A25,'Line items'!$F$2:$F$25,$C25)</f>
-        <v>19918.08</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K25" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L25" s="7" t="s">
-        <v>47</v>
-      </c>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>66</v>
       </c>
       <c r="E26" s="9" t="n">
         <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A26,'Line items'!$F$2:$F$25,$C26)</f>
-        <v>2016</v>
+        <v>19152</v>
       </c>
       <c r="F26" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A26,'Line items'!$F$2:$F$25,$C26)</f>
-        <v>1149.12</v>
+        <v>11299.68</v>
       </c>
       <c r="G26" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A26,'Line items'!$F$2:$F$25,$C26)</f>
-        <v>1219.04</v>
+        <v>11688.8</v>
       </c>
       <c r="H26" s="10" t="n">
         <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A26,'Line items'!$F$2:$F$25,$C26)</f>
+        <v>19918.08</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A27,'Line items'!$F$2:$F$25,$C27)</f>
+        <v>2016</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A27,'Line items'!$F$2:$F$25,$C27)</f>
+        <v>1149.12</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A27,'Line items'!$F$2:$F$25,$C27)</f>
+        <v>1219.04</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A27,'Line items'!$F$2:$F$25,$C27)</f>
         <v>5140.8</v>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L26" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="18" t="n">
-        <f aca="false">SUM(E25:E26)</f>
+      <c r="I27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <f aca="false">SUM(E26:E27)</f>
         <v>21168</v>
       </c>
-      <c r="F27" s="19" t="n">
-        <f aca="false">SUM(F25:F26)</f>
+      <c r="F28" s="19" t="n">
+        <f aca="false">SUM(F26:F27)</f>
         <v>12448.8</v>
       </c>
-      <c r="G27" s="19" t="n">
-        <f aca="false">SUM(G25:G26)</f>
+      <c r="G28" s="19" t="n">
+        <f aca="false">SUM(G26:G27)</f>
         <v>12907.84</v>
       </c>
-      <c r="H27" s="19" t="n">
-        <f aca="false">SUM(H25:H26)</f>
+      <c r="H28" s="19" t="n">
+        <f aca="false">SUM(H26:H27)</f>
         <v>25058.88</v>
       </c>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C28" s="8" t="s">
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A29,'Line items'!$F$2:$F$25,$C29)</f>
+        <v>43760</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A29,'Line items'!$F$2:$F$25,$C29)</f>
+        <v>957</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A29,'Line items'!$F$2:$F$25,$C29)</f>
+        <v>1274.42</v>
+      </c>
+      <c r="H29" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A29,'Line items'!$F$2:$F$25,$C29)</f>
+        <v>20830.64</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J29" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <f aca="false">SUMIFS('Line items'!H$2:H$25,'Line items'!$A$2:$A$25,$A28,'Line items'!$F$2:$F$25,$C28)</f>
+      <c r="K29" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <f aca="false">SUM(E29:E29)</f>
         <v>43760</v>
       </c>
-      <c r="F28" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!I$2:I$25,'Line items'!$A$2:$A$25,$A28,'Line items'!$F$2:$F$25,$C28)</f>
+      <c r="F30" s="19" t="n">
+        <f aca="false">SUM(F29:F29)</f>
         <v>957</v>
       </c>
-      <c r="G28" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!J$2:J$25,'Line items'!$A$2:$A$25,$A28,'Line items'!$F$2:$F$25,$C28)</f>
+      <c r="G30" s="19" t="n">
+        <f aca="false">SUM(G29:G29)</f>
         <v>1274.42</v>
       </c>
-      <c r="H28" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!K$2:K$25,'Line items'!$A$2:$A$25,$A28,'Line items'!$F$2:$F$25,$C28)</f>
+      <c r="H30" s="19" t="n">
+        <f aca="false">SUM(H29:H29)</f>
         <v>20830.64</v>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L28" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <f aca="false">SUM(E28:E28)</f>
-        <v>43760</v>
-      </c>
-      <c r="F29" s="19" t="n">
-        <f aca="false">SUM(F28:F28)</f>
-        <v>957</v>
-      </c>
-      <c r="G29" s="19" t="n">
-        <f aca="false">SUM(G28:G28)</f>
-        <v>1274.42</v>
-      </c>
-      <c r="H29" s="19" t="n">
-        <f aca="false">SUM(H28:H28)</f>
-        <v>20830.64</v>
-      </c>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="E30" s="22" t="n">
-        <f aca="false">E24+E27+E29</f>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <f aca="false">E25+E28+E30</f>
         <v>1389088</v>
       </c>
-      <c r="F30" s="23" t="n">
-        <f aca="false">F24+F27+F29</f>
+      <c r="F31" s="23" t="n">
+        <f aca="false">F25+F28+F30</f>
         <v>22979.85</v>
       </c>
-      <c r="G30" s="23" t="n">
-        <f aca="false">G24+G27+G29</f>
+      <c r="G31" s="23" t="n">
+        <f aca="false">G25+G28+G30</f>
         <v>24133</v>
       </c>
-      <c r="H30" s="23" t="n">
-        <f aca="false">H24+H27+H29</f>
+      <c r="H31" s="23" t="n">
+        <f aca="false">H25+H28+H30</f>
         <v>119371.08</v>
       </c>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B33" s="24" t="n">
-        <f aca="false">E30</f>
-        <v>1389088</v>
-      </c>
-      <c r="C33" s="24" t="n">
-        <v>1389088</v>
-      </c>
-      <c r="D33" s="24" t="n">
-        <f aca="false">B33-C33</f>
-        <v>0</v>
+      <c r="D33" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" s="24" t="n">
-        <f aca="false">F30</f>
-        <v>22979.85</v>
+        <f aca="false">E31</f>
+        <v>1389088</v>
       </c>
       <c r="C34" s="24" t="n">
-        <v>22979.85</v>
+        <v>1389088</v>
       </c>
       <c r="D34" s="24" t="n">
         <f aca="false">B34-C34</f>
@@ -1914,14 +1912,14 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B35" s="24" t="n">
-        <f aca="false">G30</f>
-        <v>24133</v>
+        <f aca="false">F31</f>
+        <v>22979.85</v>
       </c>
       <c r="C35" s="24" t="n">
-        <v>24133</v>
+        <v>22979.85</v>
       </c>
       <c r="D35" s="24" t="n">
         <f aca="false">B35-C35</f>
@@ -1930,17 +1928,33 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B36" s="24" t="n">
-        <f aca="false">H30</f>
-        <v>119371.08</v>
+        <f aca="false">G31</f>
+        <v>24133</v>
       </c>
       <c r="C36" s="24" t="n">
-        <v>119371.08</v>
+        <v>24133</v>
       </c>
       <c r="D36" s="24" t="n">
         <f aca="false">B36-C36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="24" t="n">
+        <f aca="false">H31</f>
+        <v>119371.08</v>
+      </c>
+      <c r="C37" s="24" t="n">
+        <v>119371.08</v>
+      </c>
+      <c r="D37" s="24" t="n">
+        <f aca="false">B37-C37</f>
         <v>0</v>
       </c>
     </row>
@@ -1976,60 +1990,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G1" s="25" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H1" s="25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C2" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H2" s="28" t="n">
         <v>65000</v>
@@ -2046,25 +2060,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C3" s="26" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H3" s="28" t="n">
         <v>35000</v>
@@ -2081,25 +2095,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C4" s="26" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="E4" s="26" t="s">
-        <v>95</v>
-      </c>
       <c r="F4" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H4" s="28" t="n">
         <v>32400</v>
@@ -2116,25 +2130,25 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="E5" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="F5" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="H5" s="28" t="n">
         <v>25000</v>
@@ -2151,25 +2165,25 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H6" s="28" t="n">
         <v>5600</v>
@@ -2186,25 +2200,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="E7" s="26" t="s">
-        <v>100</v>
-      </c>
       <c r="F7" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H7" s="28" t="n">
         <v>72000</v>
@@ -2221,25 +2235,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>19</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H8" s="28" t="n">
         <v>8000</v>
@@ -2256,25 +2270,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>7</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H9" s="28" t="n">
         <v>960</v>
@@ -2291,25 +2305,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>8</v>
       </c>
       <c r="D10" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="26" t="s">
-        <v>106</v>
-      </c>
       <c r="F10" s="27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H10" s="28" t="n">
         <v>2000</v>
@@ -2326,25 +2340,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>17</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H11" s="28" t="n">
         <v>5000</v>
@@ -2361,25 +2375,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>18</v>
       </c>
       <c r="D12" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="E12" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="E12" s="26" t="s">
-        <v>110</v>
-      </c>
       <c r="F12" s="27" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" s="28" t="n">
         <v>2000</v>
@@ -2396,25 +2410,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>9</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H13" s="28" t="n">
         <v>210000</v>
@@ -2431,25 +2445,25 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>10</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H14" s="28" t="n">
         <v>75000</v>
@@ -2466,25 +2480,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>11</v>
       </c>
       <c r="D15" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="E15" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="E15" s="26" t="s">
-        <v>116</v>
-      </c>
       <c r="F15" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H15" s="28" t="n">
         <v>125000</v>
@@ -2501,25 +2515,25 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>12</v>
       </c>
       <c r="D16" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" s="7" t="s">
         <v>119</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="F16" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>117</v>
       </c>
       <c r="H16" s="28" t="n">
         <v>200000</v>
@@ -2536,25 +2550,25 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C17" s="26" t="n">
         <v>13</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H17" s="28" t="n">
         <v>200000</v>
@@ -2571,25 +2585,25 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C18" s="26" t="n">
         <v>14</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E18" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H18" s="28" t="n">
         <v>180000</v>
@@ -2606,25 +2620,25 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C19" s="26" t="n">
         <v>15</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E19" s="26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H19" s="28" t="n">
         <v>30000</v>
@@ -2641,25 +2655,25 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C20" s="26" t="n">
         <v>16</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H20" s="28" t="n">
         <v>51200</v>
@@ -2676,25 +2690,25 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C21" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F21" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H21" s="28" t="n">
         <v>19152</v>
@@ -2711,25 +2725,25 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C22" s="26" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F22" s="27" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H22" s="28" t="n">
         <v>2016</v>
@@ -2746,25 +2760,25 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C23" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H23" s="28" t="n">
         <v>33600</v>
@@ -2781,25 +2795,25 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C24" s="26" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H24" s="28" t="n">
         <v>2160</v>
@@ -2816,25 +2830,25 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C25" s="26" t="n">
         <v>3</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H25" s="28" t="n">
         <v>8000</v>
@@ -2857,7 +2871,7 @@
       <c r="E26" s="20"/>
       <c r="F26" s="20"/>
       <c r="G26" s="21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H26" s="22" t="n">
         <f aca="false">SUM(H2:H25)</f>
@@ -2904,205 +2918,205 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C13" s="32" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C16" s="32" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -3130,71 +3144,71 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,10 +3217,10 @@
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>